<commit_message>
fix: 2026-07-19 엑셀 필터 활성화
</commit_message>
<xml_diff>
--- a/outputs/2026-07-19-photo-next-project-intake/photo-next-project-intake-template.xlsx
+++ b/outputs/2026-07-19-photo-next-project-intake/photo-next-project-intake-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로젝트_입력" sheetId="1" r:id="Rac22edac79e743d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성_가이드" sheetId="2" r:id="R8ac5c77a9ebd4524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="태그_목록" sheetId="3" r:id="R55ec54b12df94ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로젝트_입력" sheetId="1" r:id="R37d203501aba4df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성_가이드" sheetId="2" r:id="Ra4205f2f835d492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="태그_목록" sheetId="3" r:id="R854a071740de42ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -279,6 +279,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProjectIntakeTable" displayName="ProjectIntakeTable" ref="A1:U2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:U2"/>
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="프로젝트키"/>
     <x:tableColumn id="2" name="구분"/>
@@ -1871,7 +1872,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77e5881f314c47c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d5253b01344258"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
fix: 2026-07-19 입력 검증 정정
</commit_message>
<xml_diff>
--- a/outputs/2026-07-19-photo-next-project-intake/photo-next-project-intake-template.xlsx
+++ b/outputs/2026-07-19-photo-next-project-intake/photo-next-project-intake-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로젝트_입력" sheetId="1" r:id="R37d203501aba4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성_가이드" sheetId="2" r:id="Ra4205f2f835d492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="태그_목록" sheetId="3" r:id="R854a071740de42ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="프로젝트_입력" sheetId="1" r:id="R0a65211df77d437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성_가이드" sheetId="2" r:id="Rede2fc83e6bd41a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="태그_목록" sheetId="3" r:id="Re8463473585a47e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -27,7 +27,7 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:color rgb="FF404040"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -47,8 +47,14 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -57,7 +63,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F4E78"/>
+        <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -68,6 +74,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF8E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -156,7 +167,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -223,8 +234,9 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -242,26 +254,27 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1855,15 +1868,15 @@
       <x:formula1>"documentary,art_photo,commercial,video"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="date" operator="between" sqref="E2:F200">
-      <x:formula1>2000-01-01</x:formula1>
-      <x:formula2>2100-12-31</x:formula2>
+      <x:formula1>DATE(2000,1,1)</x:formula1>
+      <x:formula2>DATE(2100,12,31)</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="date" operator="between" sqref="S2:S200">
-      <x:formula1>2000-01-01</x:formula1>
-      <x:formula2>2100-12-31</x:formula2>
+      <x:formula1>DATE(2000,1,1)</x:formula1>
+      <x:formula2>DATE(2100,12,31)</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="custom" sqref="R2:R200">
-      <x:formula1>OR(R2="",LEFT(R2,8)="https://")</x:formula1>
+      <x:formula1>AND(R2&lt;&gt;"",LEFT(R2,8)="https://",LEN(R2)&gt;8,ISNUMBER(FIND(".",LEFT(MID(R2,9,LEN(R2)-8),FIND("/",MID(R2,9,LEN(R2)-8)&amp;"/")-1))))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="U2:U200">
       <x:formula1>0</x:formula1>
@@ -1872,7 +1885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d5253b01344258"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R682d9289eec84655"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1889,174 +1902,174 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="29" t="str">
+      <x:c r="A1" s="30" t="str">
         <x:v>PHOTO:NEXT 프로젝트 입력 가이드</x:v>
       </x:c>
-      <x:c r="B1" s="29"/>
-      <x:c r="C1" s="29"/>
-      <x:c r="D1" s="29"/>
-      <x:c r="E1" s="29"/>
+      <x:c r="B1" s="30"/>
+      <x:c r="C1" s="30"/>
+      <x:c r="D1" s="30"/>
+      <x:c r="E1" s="30"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="32" t="str">
+      <x:c r="A3" s="33" t="str">
         <x:v>입력 원칙</x:v>
       </x:c>
-      <x:c r="B3" s="33" t="str">
+      <x:c r="B3" s="34" t="str">
         <x:v>내용</x:v>
       </x:c>
-      <x:c r="C3" s="33" t="str"/>
-      <x:c r="D3" s="33" t="str"/>
-      <x:c r="E3" s="34" t="str"/>
+      <x:c r="C3" s="34" t="str"/>
+      <x:c r="D3" s="34" t="str"/>
+      <x:c r="E3" s="35" t="str"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
-      <x:c r="A4" s="38" t="str">
+      <x:c r="A4" s="39" t="str">
         <x:v>한 행 = 한 프로젝트</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="38" t="str">
         <x:v>한 프로젝트를 한 행에 입력합니다. 여러 태그·교수명·보조트랙은 세미콜론(;)으로 구분합니다.</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str"/>
-      <x:c r="D4" s="37" t="str"/>
-      <x:c r="E4" s="37" t="str"/>
+      <x:c r="C4" s="38" t="str"/>
+      <x:c r="D4" s="38" t="str"/>
+      <x:c r="E4" s="38" t="str"/>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
-      <x:c r="A5" s="38" t="str">
-        <x:v>필수 항목</x:v>
-      </x:c>
-      <x:c r="B5" s="37" t="str">
-        <x:v>파란색 헤더 열은 반드시 채웁니다. 프로젝트키는 영문 소문자·숫자·밑줄만 사용하고 중복하지 않습니다.</x:v>
-      </x:c>
-      <x:c r="C5" s="37" t="str"/>
-      <x:c r="D5" s="37" t="str"/>
-      <x:c r="E5" s="37" t="str"/>
+      <x:c r="A5" s="39" t="str">
+        <x:v>필수 열</x:v>
+      </x:c>
+      <x:c r="B5" s="38" t="str">
+        <x:v>필수 열은 연한 파란색 헤더로 표시합니다.</x:v>
+      </x:c>
+      <x:c r="C5" s="38" t="str"/>
+      <x:c r="D5" s="38" t="str"/>
+      <x:c r="E5" s="38" t="str"/>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
-      <x:c r="A6" s="38" t="str">
+      <x:c r="A6" s="39" t="str">
         <x:v>날짜</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="str">
+      <x:c r="B6" s="38" t="str">
         <x:v>시작일·종료일은 실제 행사 기간입니다. 출처확인일은 공식 게시물의 수정일 또는 검증일입니다.</x:v>
       </x:c>
-      <x:c r="C6" s="37" t="str"/>
-      <x:c r="D6" s="37" t="str"/>
-      <x:c r="E6" s="37" t="str"/>
+      <x:c r="C6" s="38" t="str"/>
+      <x:c r="D6" s="38" t="str"/>
+      <x:c r="E6" s="38" t="str"/>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
-      <x:c r="A7" s="38" t="str">
+      <x:c r="A7" s="39" t="str">
         <x:v>출처 URL</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="str">
+      <x:c r="B7" s="38" t="str">
         <x:v>공개 가능한 HTTPS 공식 페이지 주소를 입력합니다.</x:v>
       </x:c>
-      <x:c r="C7" s="37" t="str"/>
-      <x:c r="D7" s="37" t="str"/>
-      <x:c r="E7" s="37" t="str"/>
+      <x:c r="C7" s="38" t="str"/>
+      <x:c r="D7" s="38" t="str"/>
+      <x:c r="E7" s="38" t="str"/>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
-      <x:c r="A8" s="38" t="str">
+      <x:c r="A8" s="39" t="str">
         <x:v>태그</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="str">
+      <x:c r="B8" s="38" t="str">
         <x:v>대표트랙은 정확히 하나, 관심태그는 태그_목록의 키를 사용합니다. 한 행 안의 태그는 중복하지 않습니다.</x:v>
       </x:c>
-      <x:c r="C8" s="37" t="str"/>
-      <x:c r="D8" s="37" t="str"/>
-      <x:c r="E8" s="37" t="str"/>
+      <x:c r="C8" s="38" t="str"/>
+      <x:c r="D8" s="38" t="str"/>
+      <x:c r="E8" s="38" t="str"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="40" t="str">
+      <x:c r="A10" s="42" t="str">
         <x:v>입력 진행상태</x:v>
       </x:c>
-      <x:c r="B10" s="40" t="str">
+      <x:c r="B10" s="42" t="str">
         <x:v>DB 상태</x:v>
       </x:c>
-      <x:c r="C10" s="40" t="str">
+      <x:c r="C10" s="42" t="str">
         <x:v>근거 상태</x:v>
       </x:c>
-      <x:c r="D10" s="40" t="str">
+      <x:c r="D10" s="42" t="str">
         <x:v>공개 범위</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="35" t="str">
+      <x:c r="A11" s="36" t="str">
         <x:v>완료</x:v>
       </x:c>
-      <x:c r="B11" s="35" t="str">
+      <x:c r="B11" s="36" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="C11" s="35" t="str">
+      <x:c r="C11" s="36" t="str">
         <x:v>historical</x:v>
       </x:c>
-      <x:c r="D11" s="35" t="str">
+      <x:c r="D11" s="36" t="str">
         <x:v>public</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="35" t="str">
+      <x:c r="A12" s="36" t="str">
         <x:v>진행중</x:v>
       </x:c>
-      <x:c r="B12" s="35" t="str">
+      <x:c r="B12" s="36" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="C12" s="35" t="str">
+      <x:c r="C12" s="36" t="str">
         <x:v>snapshot</x:v>
       </x:c>
-      <x:c r="D12" s="35" t="str">
+      <x:c r="D12" s="36" t="str">
         <x:v>public</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="35" t="str">
+      <x:c r="A13" s="36" t="str">
         <x:v>예정확정</x:v>
       </x:c>
-      <x:c r="B13" s="35" t="str">
+      <x:c r="B13" s="36" t="str">
         <x:v>해당 연도 active / 다음 학년 next_year_confirmed</x:v>
       </x:c>
-      <x:c r="C13" s="35" t="str">
+      <x:c r="C13" s="36" t="str">
         <x:v>snapshot</x:v>
       </x:c>
-      <x:c r="D13" s="35" t="str">
+      <x:c r="D13" s="36" t="str">
         <x:v>public</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="35" t="str">
+      <x:c r="A14" s="36" t="str">
         <x:v>반복운영</x:v>
       </x:c>
-      <x:c r="B14" s="35" t="str">
+      <x:c r="B14" s="36" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="C14" s="35" t="str">
+      <x:c r="C14" s="36" t="str">
         <x:v>recurring</x:v>
       </x:c>
-      <x:c r="D14" s="35" t="str">
+      <x:c r="D14" s="36" t="str">
         <x:v>public</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="35" t="str">
+      <x:c r="A15" s="36" t="str">
         <x:v>확인필요</x:v>
       </x:c>
-      <x:c r="B15" s="35" t="str">
+      <x:c r="B15" s="36" t="str">
         <x:v>draft</x:v>
       </x:c>
-      <x:c r="C15" s="35" t="str">
+      <x:c r="C15" s="36" t="str">
         <x:v>verify_required</x:v>
       </x:c>
-      <x:c r="D15" s="35" t="str">
+      <x:c r="D15" s="36" t="str">
         <x:v>admin_only</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="40" customHeight="1">
-      <x:c r="A17" s="48" t="str">
+      <x:c r="A17" s="50" t="str">
         <x:v>검수 흐름</x:v>
       </x:c>
-      <x:c r="B17" s="46" t="str">
+      <x:c r="B17" s="48" t="str">
         <x:v>프로젝트키·필수값·날짜·URL·태그 중복을 확인한 뒤, 진행상태 변환과 요약문 검수를 거쳐 공개합니다.</x:v>
       </x:c>
-      <x:c r="C17" s="46" t="str"/>
-      <x:c r="D17" s="46" t="str"/>
-      <x:c r="E17" s="47" t="str"/>
+      <x:c r="C17" s="48" t="str"/>
+      <x:c r="D17" s="48" t="str"/>
+      <x:c r="E17" s="49" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2083,599 +2096,599 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="28" t="str">
+      <x:c r="A1" s="29" t="str">
         <x:v>PHOTO:NEXT 대표트랙 및 설문 관심태그</x:v>
       </x:c>
-      <x:c r="B1" s="28"/>
-      <x:c r="C1" s="28"/>
+      <x:c r="B1" s="29"/>
+      <x:c r="C1" s="29"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="50" t="str">
+      <x:c r="A3" s="52" t="str">
         <x:v>대표트랙 키</x:v>
       </x:c>
-      <x:c r="B3" s="50" t="str">
+      <x:c r="B3" s="52" t="str">
         <x:v>한국어 의미</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="35" t="str">
+      <x:c r="A4" s="36" t="str">
         <x:v>documentary</x:v>
       </x:c>
-      <x:c r="B4" s="35" t="str">
+      <x:c r="B4" s="36" t="str">
         <x:v>다큐멘터리 사진</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="35" t="str">
+      <x:c r="A5" s="36" t="str">
         <x:v>art_photo</x:v>
       </x:c>
-      <x:c r="B5" s="35" t="str">
+      <x:c r="B5" s="36" t="str">
         <x:v>예술사진</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="35" t="str">
+      <x:c r="A6" s="36" t="str">
         <x:v>commercial</x:v>
       </x:c>
-      <x:c r="B6" s="35" t="str">
+      <x:c r="B6" s="36" t="str">
         <x:v>광고사진</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="35" t="str">
+      <x:c r="A7" s="36" t="str">
         <x:v>video</x:v>
       </x:c>
-      <x:c r="B7" s="35" t="str">
+      <x:c r="B7" s="36" t="str">
         <x:v>영상과 기술</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="50" t="str">
+      <x:c r="A9" s="52" t="str">
         <x:v>관심태그 키</x:v>
       </x:c>
-      <x:c r="B9" s="50" t="str">
+      <x:c r="B9" s="52" t="str">
         <x:v>한국어 의미</x:v>
       </x:c>
-      <x:c r="C9" s="50" t="str">
+      <x:c r="C9" s="52" t="str">
         <x:v>연결 설문 범주</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="36" t="str">
+      <x:c r="A10" s="37" t="str">
         <x:v>art_photo</x:v>
       </x:c>
-      <x:c r="B10" s="36" t="str">
+      <x:c r="B10" s="37" t="str">
         <x:v>예술사진</x:v>
       </x:c>
-      <x:c r="C10" s="36" t="str">
+      <x:c r="C10" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="36" t="str">
+      <x:c r="A11" s="37" t="str">
         <x:v>brand</x:v>
       </x:c>
-      <x:c r="B11" s="36" t="str">
+      <x:c r="B11" s="37" t="str">
         <x:v>브랜드</x:v>
       </x:c>
-      <x:c r="C11" s="36" t="str">
+      <x:c r="C11" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="36" t="str">
+      <x:c r="A12" s="37" t="str">
         <x:v>camera</x:v>
       </x:c>
-      <x:c r="B12" s="36" t="str">
+      <x:c r="B12" s="37" t="str">
         <x:v>카메라</x:v>
       </x:c>
-      <x:c r="C12" s="36" t="str">
+      <x:c r="C12" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="36" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>cinematography</x:v>
       </x:c>
-      <x:c r="B13" s="36" t="str">
+      <x:c r="B13" s="37" t="str">
         <x:v>영상촬영</x:v>
       </x:c>
-      <x:c r="C13" s="36" t="str">
+      <x:c r="C13" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="36" t="str">
+      <x:c r="A14" s="37" t="str">
         <x:v>collaboration</x:v>
       </x:c>
-      <x:c r="B14" s="36" t="str">
+      <x:c r="B14" s="37" t="str">
         <x:v>협업</x:v>
       </x:c>
-      <x:c r="C14" s="36" t="str">
+      <x:c r="C14" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="36" t="str">
+      <x:c r="A15" s="37" t="str">
         <x:v>color_grading</x:v>
       </x:c>
-      <x:c r="B15" s="36" t="str">
+      <x:c r="B15" s="37" t="str">
         <x:v>색보정</x:v>
       </x:c>
-      <x:c r="C15" s="36" t="str">
+      <x:c r="C15" s="37" t="str">
         <x:v>활동 선호, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="36" t="str">
+      <x:c r="A16" s="37" t="str">
         <x:v>commercial</x:v>
       </x:c>
-      <x:c r="B16" s="36" t="str">
+      <x:c r="B16" s="37" t="str">
         <x:v>광고사진</x:v>
       </x:c>
-      <x:c r="C16" s="36" t="str">
+      <x:c r="C16" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="36" t="str">
+      <x:c r="A17" s="37" t="str">
         <x:v>content</x:v>
       </x:c>
-      <x:c r="B17" s="36" t="str">
+      <x:c r="B17" s="37" t="str">
         <x:v>콘텐츠</x:v>
       </x:c>
-      <x:c r="C17" s="36" t="str">
+      <x:c r="C17" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="36" t="str">
+      <x:c r="A18" s="37" t="str">
         <x:v>cultural_planning</x:v>
       </x:c>
-      <x:c r="B18" s="36" t="str">
+      <x:c r="B18" s="37" t="str">
         <x:v>문화기획</x:v>
       </x:c>
-      <x:c r="C18" s="36" t="str">
+      <x:c r="C18" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="36" t="str">
+      <x:c r="A19" s="37" t="str">
         <x:v>daily_life</x:v>
       </x:c>
-      <x:c r="B19" s="36" t="str">
+      <x:c r="B19" s="37" t="str">
         <x:v>일상</x:v>
       </x:c>
-      <x:c r="C19" s="36" t="str">
+      <x:c r="C19" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="36" t="str">
+      <x:c r="A20" s="37" t="str">
         <x:v>digital_image</x:v>
       </x:c>
-      <x:c r="B20" s="36" t="str">
+      <x:c r="B20" s="37" t="str">
         <x:v>디지털이미지</x:v>
       </x:c>
-      <x:c r="C20" s="36" t="str">
+      <x:c r="C20" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="36" t="str">
+      <x:c r="A21" s="37" t="str">
         <x:v>documentary</x:v>
       </x:c>
-      <x:c r="B21" s="36" t="str">
+      <x:c r="B21" s="37" t="str">
         <x:v>다큐멘터리</x:v>
       </x:c>
-      <x:c r="C21" s="36" t="str">
+      <x:c r="C21" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="36" t="str">
+      <x:c r="A22" s="37" t="str">
         <x:v>editing</x:v>
       </x:c>
-      <x:c r="B22" s="36" t="str">
+      <x:c r="B22" s="37" t="str">
         <x:v>편집</x:v>
       </x:c>
-      <x:c r="C22" s="36" t="str">
+      <x:c r="C22" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="36" t="str">
+      <x:c r="A23" s="37" t="str">
         <x:v>exhibition</x:v>
       </x:c>
-      <x:c r="B23" s="36" t="str">
+      <x:c r="B23" s="37" t="str">
         <x:v>전시</x:v>
       </x:c>
-      <x:c r="C23" s="36" t="str">
+      <x:c r="C23" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="36" t="str">
+      <x:c r="A24" s="37" t="str">
         <x:v>exploration</x:v>
       </x:c>
-      <x:c r="B24" s="36" t="str">
+      <x:c r="B24" s="37" t="str">
         <x:v>탐색</x:v>
       </x:c>
-      <x:c r="C24" s="36" t="str">
+      <x:c r="C24" s="37" t="str">
         <x:v>진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="36" t="str">
+      <x:c r="A25" s="37" t="str">
         <x:v>fashion</x:v>
       </x:c>
-      <x:c r="B25" s="36" t="str">
+      <x:c r="B25" s="37" t="str">
         <x:v>패션</x:v>
       </x:c>
-      <x:c r="C25" s="36" t="str">
+      <x:c r="C25" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="36" t="str">
+      <x:c r="A26" s="37" t="str">
         <x:v>field</x:v>
       </x:c>
-      <x:c r="B26" s="36" t="str">
+      <x:c r="B26" s="37" t="str">
         <x:v>현장</x:v>
       </x:c>
-      <x:c r="C26" s="36" t="str">
+      <x:c r="C26" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="36" t="str">
+      <x:c r="A27" s="37" t="str">
         <x:v>freelance</x:v>
       </x:c>
-      <x:c r="B27" s="36" t="str">
+      <x:c r="B27" s="37" t="str">
         <x:v>프리랜서</x:v>
       </x:c>
-      <x:c r="C27" s="36" t="str">
+      <x:c r="C27" s="37" t="str">
         <x:v>진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="36" t="str">
+      <x:c r="A28" s="37" t="str">
         <x:v>installation</x:v>
       </x:c>
-      <x:c r="B28" s="36" t="str">
+      <x:c r="B28" s="37" t="str">
         <x:v>설치작업</x:v>
       </x:c>
-      <x:c r="C28" s="36" t="str">
+      <x:c r="C28" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="36" t="str">
+      <x:c r="A29" s="37" t="str">
         <x:v>interview</x:v>
       </x:c>
-      <x:c r="B29" s="36" t="str">
+      <x:c r="B29" s="37" t="str">
         <x:v>인터뷰</x:v>
       </x:c>
-      <x:c r="C29" s="36" t="str">
+      <x:c r="C29" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="36" t="str">
+      <x:c r="A30" s="37" t="str">
         <x:v>landscape</x:v>
       </x:c>
-      <x:c r="B30" s="36" t="str">
+      <x:c r="B30" s="37" t="str">
         <x:v>풍경</x:v>
       </x:c>
-      <x:c r="C30" s="36" t="str">
+      <x:c r="C30" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="36" t="str">
+      <x:c r="A31" s="37" t="str">
         <x:v>lighting</x:v>
       </x:c>
-      <x:c r="B31" s="36" t="str">
+      <x:c r="B31" s="37" t="str">
         <x:v>조명</x:v>
       </x:c>
-      <x:c r="C31" s="36" t="str">
+      <x:c r="C31" s="37" t="str">
         <x:v>활동 선호, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="36" t="str">
+      <x:c r="A32" s="37" t="str">
         <x:v>local_culture</x:v>
       </x:c>
-      <x:c r="B32" s="36" t="str">
+      <x:c r="B32" s="37" t="str">
         <x:v>지역문화</x:v>
       </x:c>
-      <x:c r="C32" s="36" t="str">
+      <x:c r="C32" s="37" t="str">
         <x:v>활동 선호, 작업 방식, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="36" t="str">
+      <x:c r="A33" s="37" t="str">
         <x:v>media_art</x:v>
       </x:c>
-      <x:c r="B33" s="36" t="str">
+      <x:c r="B33" s="37" t="str">
         <x:v>미디어아트</x:v>
       </x:c>
-      <x:c r="C33" s="36" t="str">
+      <x:c r="C33" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="36" t="str">
+      <x:c r="A34" s="37" t="str">
         <x:v>music_video</x:v>
       </x:c>
-      <x:c r="B34" s="36" t="str">
+      <x:c r="B34" s="37" t="str">
         <x:v>뮤직비디오</x:v>
       </x:c>
-      <x:c r="C34" s="36" t="str">
+      <x:c r="C34" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="36" t="str">
+      <x:c r="A35" s="37" t="str">
         <x:v>oral_history</x:v>
       </x:c>
-      <x:c r="B35" s="36" t="str">
+      <x:c r="B35" s="37" t="str">
         <x:v>구술기록</x:v>
       </x:c>
-      <x:c r="C35" s="36" t="str">
+      <x:c r="C35" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="36" t="str">
+      <x:c r="A36" s="37" t="str">
         <x:v>people</x:v>
       </x:c>
-      <x:c r="B36" s="36" t="str">
+      <x:c r="B36" s="37" t="str">
         <x:v>인물</x:v>
       </x:c>
-      <x:c r="C36" s="36" t="str">
+      <x:c r="C36" s="37" t="str">
         <x:v>활동 선호, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="36" t="str">
+      <x:c r="A37" s="37" t="str">
         <x:v>photobook</x:v>
       </x:c>
-      <x:c r="B37" s="36" t="str">
+      <x:c r="B37" s="37" t="str">
         <x:v>포토북</x:v>
       </x:c>
-      <x:c r="C37" s="36" t="str">
+      <x:c r="C37" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="36" t="str">
+      <x:c r="A38" s="37" t="str">
         <x:v>photography</x:v>
       </x:c>
-      <x:c r="B38" s="36" t="str">
+      <x:c r="B38" s="37" t="str">
         <x:v>사진</x:v>
       </x:c>
-      <x:c r="C38" s="36" t="str">
+      <x:c r="C38" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="36" t="str">
+      <x:c r="A39" s="37" t="str">
         <x:v>planning</x:v>
       </x:c>
-      <x:c r="B39" s="36" t="str">
+      <x:c r="B39" s="37" t="str">
         <x:v>기획</x:v>
       </x:c>
-      <x:c r="C39" s="36" t="str">
+      <x:c r="C39" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="36" t="str">
+      <x:c r="A40" s="37" t="str">
         <x:v>portfolio</x:v>
       </x:c>
-      <x:c r="B40" s="36" t="str">
+      <x:c r="B40" s="37" t="str">
         <x:v>포트폴리오</x:v>
       </x:c>
-      <x:c r="C40" s="36" t="str">
+      <x:c r="C40" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="36" t="str">
+      <x:c r="A41" s="37" t="str">
         <x:v>portrait</x:v>
       </x:c>
-      <x:c r="B41" s="36" t="str">
+      <x:c r="B41" s="37" t="str">
         <x:v>인물사진</x:v>
       </x:c>
-      <x:c r="C41" s="36" t="str">
+      <x:c r="C41" s="37" t="str">
         <x:v>활동 선호, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="36" t="str">
+      <x:c r="A42" s="37" t="str">
         <x:v>post_production</x:v>
       </x:c>
-      <x:c r="B42" s="36" t="str">
+      <x:c r="B42" s="37" t="str">
         <x:v>후반작업</x:v>
       </x:c>
-      <x:c r="C42" s="36" t="str">
+      <x:c r="C42" s="37" t="str">
         <x:v>활동 선호, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="36" t="str">
+      <x:c r="A43" s="37" t="str">
         <x:v>product</x:v>
       </x:c>
-      <x:c r="B43" s="36" t="str">
+      <x:c r="B43" s="37" t="str">
         <x:v>제품</x:v>
       </x:c>
-      <x:c r="C43" s="36" t="str">
+      <x:c r="C43" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="36" t="str">
+      <x:c r="A44" s="37" t="str">
         <x:v>production</x:v>
       </x:c>
-      <x:c r="B44" s="36" t="str">
+      <x:c r="B44" s="37" t="str">
         <x:v>제작</x:v>
       </x:c>
-      <x:c r="C44" s="36" t="str">
+      <x:c r="C44" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="36" t="str">
+      <x:c r="A45" s="37" t="str">
         <x:v>project</x:v>
       </x:c>
-      <x:c r="B45" s="36" t="str">
+      <x:c r="B45" s="37" t="str">
         <x:v>프로젝트</x:v>
       </x:c>
-      <x:c r="C45" s="36" t="str">
+      <x:c r="C45" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="36" t="str">
+      <x:c r="A46" s="37" t="str">
         <x:v>promotion</x:v>
       </x:c>
-      <x:c r="B46" s="36" t="str">
+      <x:c r="B46" s="37" t="str">
         <x:v>홍보</x:v>
       </x:c>
-      <x:c r="C46" s="36" t="str">
+      <x:c r="C46" s="37" t="str">
         <x:v>희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="36" t="str">
+      <x:c r="A47" s="37" t="str">
         <x:v>proposal</x:v>
       </x:c>
-      <x:c r="B47" s="36" t="str">
+      <x:c r="B47" s="37" t="str">
         <x:v>제안서</x:v>
       </x:c>
-      <x:c r="C47" s="36" t="str">
+      <x:c r="C47" s="37" t="str">
         <x:v>희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="36" t="str">
+      <x:c r="A48" s="37" t="str">
         <x:v>public_content</x:v>
       </x:c>
-      <x:c r="B48" s="36" t="str">
+      <x:c r="B48" s="37" t="str">
         <x:v>공공콘텐츠</x:v>
       </x:c>
-      <x:c r="C48" s="36" t="str">
+      <x:c r="C48" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="36" t="str">
+      <x:c r="A49" s="37" t="str">
         <x:v>research</x:v>
       </x:c>
-      <x:c r="B49" s="36" t="str">
+      <x:c r="B49" s="37" t="str">
         <x:v>리서치</x:v>
       </x:c>
-      <x:c r="C49" s="36" t="str">
+      <x:c r="C49" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="36" t="str">
+      <x:c r="A50" s="37" t="str">
         <x:v>scene</x:v>
       </x:c>
-      <x:c r="B50" s="36" t="str">
+      <x:c r="B50" s="37" t="str">
         <x:v>장면</x:v>
       </x:c>
-      <x:c r="C50" s="36" t="str">
+      <x:c r="C50" s="37" t="str">
         <x:v>활동 선호</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="36" t="str">
+      <x:c r="A51" s="37" t="str">
         <x:v>sequencing</x:v>
       </x:c>
-      <x:c r="B51" s="36" t="str">
+      <x:c r="B51" s="37" t="str">
         <x:v>시퀀싱</x:v>
       </x:c>
-      <x:c r="C51" s="36" t="str">
+      <x:c r="C51" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="36" t="str">
+      <x:c r="A52" s="37" t="str">
         <x:v>shortform</x:v>
       </x:c>
-      <x:c r="B52" s="36" t="str">
+      <x:c r="B52" s="37" t="str">
         <x:v>숏폼</x:v>
       </x:c>
-      <x:c r="C52" s="36" t="str">
+      <x:c r="C52" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="36" t="str">
+      <x:c r="A53" s="37" t="str">
         <x:v>showreel</x:v>
       </x:c>
-      <x:c r="B53" s="36" t="str">
+      <x:c r="B53" s="37" t="str">
         <x:v>쇼릴</x:v>
       </x:c>
-      <x:c r="C53" s="36" t="str">
+      <x:c r="C53" s="37" t="str">
         <x:v>희망 결과물, 진로 방향</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="36" t="str">
+      <x:c r="A54" s="37" t="str">
         <x:v>solo</x:v>
       </x:c>
-      <x:c r="B54" s="36" t="str">
+      <x:c r="B54" s="37" t="str">
         <x:v>개인작업</x:v>
       </x:c>
-      <x:c r="C54" s="36" t="str">
+      <x:c r="C54" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="36" t="str">
+      <x:c r="A55" s="37" t="str">
         <x:v>storytelling</x:v>
       </x:c>
-      <x:c r="B55" s="36" t="str">
+      <x:c r="B55" s="37" t="str">
         <x:v>스토리텔링</x:v>
       </x:c>
-      <x:c r="C55" s="36" t="str">
+      <x:c r="C55" s="37" t="str">
         <x:v>활동 선호, 희망 결과물</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="36" t="str">
+      <x:c r="A56" s="37" t="str">
         <x:v>studio</x:v>
       </x:c>
-      <x:c r="B56" s="36" t="str">
+      <x:c r="B56" s="37" t="str">
         <x:v>스튜디오</x:v>
       </x:c>
-      <x:c r="C56" s="36" t="str">
+      <x:c r="C56" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="36" t="str">
+      <x:c r="A57" s="37" t="str">
         <x:v>team</x:v>
       </x:c>
-      <x:c r="B57" s="36" t="str">
+      <x:c r="B57" s="37" t="str">
         <x:v>팀작업</x:v>
       </x:c>
-      <x:c r="C57" s="36" t="str">
+      <x:c r="C57" s="37" t="str">
         <x:v>작업 방식</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="36" t="str">
+      <x:c r="A58" s="37" t="str">
         <x:v>video</x:v>
       </x:c>
-      <x:c r="B58" s="36" t="str">
+      <x:c r="B58" s="37" t="str">
         <x:v>영상</x:v>
       </x:c>
-      <x:c r="C58" s="36" t="str">
+      <x:c r="C58" s="37" t="str">
         <x:v>활동 선호, 희망 결과물, 작업 방식, 진로 방향</x:v>
       </x:c>
     </x:row>

</xml_diff>